<commit_message>
docs: validate check-in staging configuration
</commit_message>
<xml_diff>
--- a/outputs/checkin-v1/Agendamento Line Transportes - Staging.xlsx
+++ b/outputs/checkin-v1/Agendamento Line Transportes - Staging.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form1" sheetId="1" r:id="R149d4f6605d94ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rbd8f01586d4d45e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,34 +13,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
-    <x:numFmt numFmtId="200" formatCode="0"/>
-    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm:ss"/>
-    <x:numFmt numFmtId="202" formatCode="@"/>
-  </x:numFmts>
-  <x:fonts count="2">
+  <x:fonts count="1">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="2">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF176B64"/>
-      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="1">
@@ -49,28 +33,8 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -96,13 +60,13 @@
     <x:tableColumn id="12" name="Tipo de veículo"/>
     <x:tableColumn id="13" name="Produto"/>
     <x:tableColumn id="14" name="Usina de origem"/>
-    <x:tableColumn id="15" name="Nº da(s) Nota(s) Fiscal(is) de USINA"/>
-    <x:tableColumn id="16" name="Nº da Nota Fiscal de Remessa"/>
+    <x:tableColumn id="15" name="Nº da(s) Nota(s) Fiscal(is) de USINA "/>
+    <x:tableColumn id="16" name="Nº da Nota Fiscal de Remessa"/>
     <x:tableColumn id="17" name="Estou ciente de que, após concluir o check-in, devo enviar a foto da NF de Usina para o WhatsApp da Line Transportes: (13) 99652-4561."/>
     <x:tableColumn id="18" name="Estou ciente de que o check-in confirma somente minha chegada à Baixada Santista, não garante posição ou ordem de descarga, e devo aguardar o contato da Line por telefone ou WhatsApp."/>
     <x:tableColumn id="19" name="Identificador de check-in"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -301,90 +265,72 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="27" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="29" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="42" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="86" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Id</x:v>
       </x:c>
-      <x:c r="B1" s="7" t="str">
+      <x:c r="B1" t="str">
         <x:v>Start time</x:v>
       </x:c>
-      <x:c r="C1" s="7" t="str">
+      <x:c r="C1" t="str">
         <x:v>Completion time</x:v>
       </x:c>
-      <x:c r="D1" s="8" t="str">
+      <x:c r="D1" t="str">
         <x:v>Email</x:v>
       </x:c>
-      <x:c r="E1" s="8" t="str">
+      <x:c r="E1" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="F1" s="8" t="str">
+      <x:c r="F1" t="str">
         <x:v>Language</x:v>
       </x:c>
-      <x:c r="G1" s="8" t="str">
+      <x:c r="G1" t="str">
         <x:v>Nome completo do motorista</x:v>
       </x:c>
-      <x:c r="H1" s="8" t="str">
+      <x:c r="H1" t="str">
         <x:v>CNH do motorista</x:v>
       </x:c>
-      <x:c r="I1" s="8" t="str">
+      <x:c r="I1" t="str">
         <x:v>Telefone do motorista (com DDD)</x:v>
       </x:c>
-      <x:c r="J1" s="8" t="str">
+      <x:c r="J1" t="str">
         <x:v>Placa</x:v>
       </x:c>
-      <x:c r="K1" s="8" t="str">
+      <x:c r="K1" t="str">
         <x:v>Nome da Transportadora</x:v>
       </x:c>
-      <x:c r="L1" s="8" t="str">
+      <x:c r="L1" t="str">
         <x:v>Tipo de veículo</x:v>
       </x:c>
-      <x:c r="M1" s="8" t="str">
+      <x:c r="M1" t="str">
         <x:v>Produto</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" t="str">
         <x:v>Usina de origem</x:v>
       </x:c>
-      <x:c r="O1" s="8" t="str">
-        <x:v>Nº da(s) Nota(s) Fiscal(is) de USINA</x:v>
-      </x:c>
-      <x:c r="P1" s="8" t="str">
-        <x:v>Nº da Nota Fiscal de Remessa</x:v>
-      </x:c>
-      <x:c r="Q1" s="8" t="str">
+      <x:c r="O1" t="str">
+        <x:v>Nº da(s) Nota(s) Fiscal(is) de USINA </x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>Nº da Nota Fiscal de Remessa</x:v>
+      </x:c>
+      <x:c r="Q1" t="str">
         <x:v>Estou ciente de que, após concluir o check-in, devo enviar a foto da NF de Usina para o WhatsApp da Line Transportes: (13) 99652-4561.</x:v>
       </x:c>
-      <x:c r="R1" s="8" t="str">
+      <x:c r="R1" t="str">
         <x:v>Estou ciente de que o check-in confirma somente minha chegada à Baixada Santista, não garante posição ou ordem de descarga, e devo aguardar o contato da Line por telefone ou WhatsApp.</x:v>
       </x:c>
-      <x:c r="S1" s="8" t="str">
+      <x:c r="S1" t="str">
         <x:v>Identificador de check-in</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re42eb27fca0a4a44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R768fcc4c25a440af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>